<commit_message>
[BE](api) S15P11E102-348 fact_candidate 취소 엔드포인트 — '기억하지 마'의 서버 절반
</commit_message>
<xml_diff>
--- a/docs/database/column-definition/BOMI_컬럼정의서.xlsx
+++ b/docs/database/column-definition/BOMI_컬럼정의서.xlsx
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -807,6 +807,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -936,6 +937,28 @@
       <c r="D9" t="inlineStr">
         <is>
           <t>'오늘 날씨 어때?'의 기본 지역이 없어 로봇이 되묻거나 지어내던 문제를 없애기 위해. 로봇 대화 문맥 채널 전용이며 가디언웹에는 노출하지 않는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>fact_candidate.status 에 CANCELLED_BY_SENIOR 추가 (S15P11E102-348)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fact_candidate</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>어르신의 '기억하지 마' 요청으로 이미 제출된 미확정 후보를 닫는 상태가 없어, 지운 이야기가 재질의로 되살아날 수 있던 문제를 없애기 위해. DB CHECK 없는 varchar(40)이라 DDL 변경은 없다</t>
         </is>
       </c>
     </row>
@@ -18940,7 +18963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E223"/>
+  <dimension ref="A1:E224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -18964,6 +18987,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -22016,1458 +22040,1454 @@
       </c>
     </row>
     <row r="117" ht="15" customHeight="1">
-      <c r="A117" s="26" t="inlineStr">
+      <c r="A117" s="25" t="inlineStr">
+        <is>
+          <t>fact_candidate.status</t>
+        </is>
+      </c>
+      <c r="B117" s="25" t="inlineStr">
+        <is>
+          <t>CANCELLED_BY_SENIOR</t>
+        </is>
+      </c>
+      <c r="C117" s="25" t="inlineStr">
+        <is>
+          <t>어르신 요청 취소</t>
+        </is>
+      </c>
+      <c r="D117" s="25" t="inlineStr">
+        <is>
+          <t>어르신 본인이 '기억하지 마'로 닫은 미확정 후보. 재질의·확인요청·검색·반영에서 제외한다. REJECTED(보호자·시스템 거절)와 구분한다 — 누가 왜 닫았는지가 T4 신뢰의 근거다.</t>
+        </is>
+      </c>
+      <c r="E117" s="25" t="n"/>
+    </row>
+    <row r="118" ht="15" customHeight="1">
+      <c r="A118" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason</t>
         </is>
       </c>
-      <c r="B117" s="26" t="inlineStr">
+      <c r="B118" s="26" t="inlineStr">
         <is>
           <t>MISSING_REQUIRED_FIELD</t>
         </is>
       </c>
-      <c r="C117" s="26" t="inlineStr">
+      <c r="C118" s="26" t="inlineStr">
         <is>
           <t>재질의 사유: MISSING_REQUIRED_FIELD</t>
         </is>
       </c>
-      <c r="D117" s="26" t="inlineStr">
+      <c r="D118" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E117" s="26" t="inlineStr">
+      <c r="E118" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="15" customHeight="1">
-      <c r="A118" s="25" t="inlineStr">
+    <row r="119" ht="15" customHeight="1">
+      <c r="A119" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason</t>
         </is>
       </c>
-      <c r="B118" s="25" t="inlineStr">
+      <c r="B119" s="25" t="inlineStr">
         <is>
           <t>AMBIGUOUS_VALUE</t>
         </is>
       </c>
-      <c r="C118" s="25" t="inlineStr">
+      <c r="C119" s="25" t="inlineStr">
         <is>
           <t>재질의 사유: AMBIGUOUS_VALUE</t>
         </is>
       </c>
-      <c r="D118" s="25" t="inlineStr">
+      <c r="D119" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E118" s="25" t="inlineStr">
+      <c r="E119" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="15" customHeight="1">
-      <c r="A119" s="26" t="inlineStr">
+    <row r="120" ht="15" customHeight="1">
+      <c r="A120" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason</t>
         </is>
       </c>
-      <c r="B119" s="26" t="inlineStr">
+      <c r="B120" s="26" t="inlineStr">
         <is>
           <t>LOW_RECOGNITION_CONFIDENCE</t>
         </is>
       </c>
-      <c r="C119" s="26" t="inlineStr">
+      <c r="C120" s="26" t="inlineStr">
         <is>
           <t>재질의 사유: LOW_RECOGNITION_CONFIDENCE</t>
         </is>
       </c>
-      <c r="D119" s="26" t="inlineStr">
+      <c r="D120" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E119" s="26" t="inlineStr">
+      <c r="E120" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="15" customHeight="1">
-      <c r="A120" s="25" t="inlineStr">
+    <row r="121" ht="15" customHeight="1">
+      <c r="A121" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason</t>
         </is>
       </c>
-      <c r="B120" s="25" t="inlineStr">
+      <c r="B121" s="25" t="inlineStr">
         <is>
           <t>CONFLICT_WITH_EXISTING_DATA</t>
         </is>
       </c>
-      <c r="C120" s="25" t="inlineStr">
+      <c r="C121" s="25" t="inlineStr">
         <is>
           <t>재질의 사유: CONFLICT_WITH_EXISTING_DATA</t>
         </is>
       </c>
-      <c r="D120" s="25" t="inlineStr">
+      <c r="D121" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E120" s="25" t="inlineStr">
+      <c r="E121" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="15" customHeight="1">
-      <c r="A121" s="26" t="inlineStr">
+    <row r="122" ht="15" customHeight="1">
+      <c r="A122" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason</t>
         </is>
       </c>
-      <c r="B121" s="26" t="inlineStr">
+      <c r="B122" s="26" t="inlineStr">
         <is>
           <t>SENSITIVE_INFORMATION_CONFIRMATION</t>
         </is>
       </c>
-      <c r="C121" s="26" t="inlineStr">
+      <c r="C122" s="26" t="inlineStr">
         <is>
           <t>재질의 사유: SENSITIVE_INFORMATION_CONFIRMATION</t>
         </is>
       </c>
-      <c r="D121" s="26" t="inlineStr">
+      <c r="D122" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.clarification_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E121" s="26" t="inlineStr">
+      <c r="E122" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="122" ht="15" customHeight="1">
-      <c r="A122" s="25" t="inlineStr">
+    <row r="123" ht="15" customHeight="1">
+      <c r="A123" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B122" s="25" t="inlineStr">
+      <c r="B123" s="25" t="inlineStr">
         <is>
           <t>NOT_REQUIRED</t>
         </is>
       </c>
-      <c r="C122" s="25" t="inlineStr">
+      <c r="C123" s="25" t="inlineStr">
         <is>
           <t>협의 상태: NOT_REQUIRED</t>
         </is>
       </c>
-      <c r="D122" s="25" t="inlineStr">
+      <c r="D123" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E122" s="25" t="inlineStr">
+      <c r="E123" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="15" customHeight="1">
-      <c r="A123" s="26" t="inlineStr">
+    <row r="124" ht="15" customHeight="1">
+      <c r="A124" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B123" s="26" t="inlineStr">
+      <c r="B124" s="26" t="inlineStr">
         <is>
           <t>COORDINATION_REQUIRED</t>
         </is>
       </c>
-      <c r="C123" s="26" t="inlineStr">
+      <c r="C124" s="26" t="inlineStr">
         <is>
           <t>협의 상태: COORDINATION_REQUIRED</t>
         </is>
       </c>
-      <c r="D123" s="26" t="inlineStr">
+      <c r="D124" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E123" s="26" t="inlineStr">
+      <c r="E124" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="15" customHeight="1">
-      <c r="A124" s="25" t="inlineStr">
+    <row r="125" ht="15" customHeight="1">
+      <c r="A125" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B124" s="25" t="inlineStr">
+      <c r="B125" s="25" t="inlineStr">
         <is>
           <t>WAITING_PRIMARY_GUARDIAN</t>
         </is>
       </c>
-      <c r="C124" s="25" t="inlineStr">
+      <c r="C125" s="25" t="inlineStr">
         <is>
           <t>협의 상태: WAITING_PRIMARY_GUARDIAN</t>
         </is>
       </c>
-      <c r="D124" s="25" t="inlineStr">
+      <c r="D125" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E124" s="25" t="inlineStr">
+      <c r="E125" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="15" customHeight="1">
-      <c r="A125" s="26" t="inlineStr">
+    <row r="126" ht="15" customHeight="1">
+      <c r="A126" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B125" s="26" t="inlineStr">
+      <c r="B126" s="26" t="inlineStr">
         <is>
           <t>WAITING_SENIOR</t>
         </is>
       </c>
-      <c r="C125" s="26" t="inlineStr">
+      <c r="C126" s="26" t="inlineStr">
         <is>
           <t>협의 상태: WAITING_SENIOR</t>
         </is>
       </c>
-      <c r="D125" s="26" t="inlineStr">
+      <c r="D126" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E125" s="26" t="inlineStr">
+      <c r="E126" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="15" customHeight="1">
-      <c r="A126" s="25" t="inlineStr">
+    <row r="127" ht="15" customHeight="1">
+      <c r="A127" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B126" s="25" t="inlineStr">
+      <c r="B127" s="25" t="inlineStr">
         <is>
           <t>AGREED</t>
         </is>
       </c>
-      <c r="C126" s="25" t="inlineStr">
+      <c r="C127" s="25" t="inlineStr">
         <is>
           <t>협의 상태: AGREED</t>
         </is>
       </c>
-      <c r="D126" s="25" t="inlineStr">
+      <c r="D127" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E126" s="25" t="inlineStr">
+      <c r="E127" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="15" customHeight="1">
-      <c r="A127" s="26" t="inlineStr">
+    <row r="128" ht="15" customHeight="1">
+      <c r="A128" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B127" s="26" t="inlineStr">
+      <c r="B128" s="26" t="inlineStr">
         <is>
           <t>DISAGREED</t>
         </is>
       </c>
-      <c r="C127" s="26" t="inlineStr">
+      <c r="C128" s="26" t="inlineStr">
         <is>
           <t>협의 상태: DISAGREED</t>
         </is>
       </c>
-      <c r="D127" s="26" t="inlineStr">
+      <c r="D128" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E127" s="26" t="inlineStr">
+      <c r="E128" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="15" customHeight="1">
-      <c r="A128" s="25" t="inlineStr">
+    <row r="129" ht="15" customHeight="1">
+      <c r="A129" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B128" s="25" t="inlineStr">
+      <c r="B129" s="25" t="inlineStr">
         <is>
           <t>SENIOR_UNREACHABLE</t>
         </is>
       </c>
-      <c r="C128" s="25" t="inlineStr">
+      <c r="C129" s="25" t="inlineStr">
         <is>
           <t>협의 상태: SENIOR_UNREACHABLE</t>
         </is>
       </c>
-      <c r="D128" s="25" t="inlineStr">
+      <c r="D129" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E128" s="25" t="inlineStr">
+      <c r="E129" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="129" ht="15" customHeight="1">
-      <c r="A129" s="26" t="inlineStr">
+    <row r="130" ht="15" customHeight="1">
+      <c r="A130" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B129" s="26" t="inlineStr">
+      <c r="B130" s="26" t="inlineStr">
         <is>
           <t>GUARDIAN_OVERRIDE_CONFIRMED</t>
         </is>
       </c>
-      <c r="C129" s="26" t="inlineStr">
+      <c r="C130" s="26" t="inlineStr">
         <is>
           <t>협의 상태: GUARDIAN_OVERRIDE_CONFIRMED</t>
         </is>
       </c>
-      <c r="D129" s="26" t="inlineStr">
+      <c r="D130" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E129" s="26" t="inlineStr">
+      <c r="E130" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="130" ht="15" customHeight="1">
-      <c r="A130" s="25" t="inlineStr">
+    <row r="131" ht="15" customHeight="1">
+      <c r="A131" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status</t>
         </is>
       </c>
-      <c r="B130" s="25" t="inlineStr">
+      <c r="B131" s="25" t="inlineStr">
         <is>
           <t>COMPLETED</t>
         </is>
       </c>
-      <c r="C130" s="25" t="inlineStr">
+      <c r="C131" s="25" t="inlineStr">
         <is>
           <t>협의 상태: COMPLETED</t>
         </is>
       </c>
-      <c r="D130" s="25" t="inlineStr">
+      <c r="D131" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.coordination_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E130" s="25" t="inlineStr">
+      <c r="E131" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="15" customHeight="1">
-      <c r="A131" s="26" t="inlineStr">
+    <row r="132" ht="15" customHeight="1">
+      <c r="A132" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position</t>
         </is>
       </c>
-      <c r="B131" s="26" t="inlineStr">
+      <c r="B132" s="26" t="inlineStr">
         <is>
           <t>NOT_REQUESTED</t>
         </is>
       </c>
-      <c r="C131" s="26" t="inlineStr">
+      <c r="C132" s="26" t="inlineStr">
         <is>
           <t>시니어 입장: NOT_REQUESTED</t>
         </is>
       </c>
-      <c r="D131" s="26" t="inlineStr">
+      <c r="D132" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E131" s="26" t="inlineStr">
+      <c r="E132" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="132" ht="15" customHeight="1">
-      <c r="A132" s="25" t="inlineStr">
+    <row r="133" ht="15" customHeight="1">
+      <c r="A133" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position</t>
         </is>
       </c>
-      <c r="B132" s="25" t="inlineStr">
+      <c r="B133" s="25" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="C132" s="25" t="inlineStr">
+      <c r="C133" s="25" t="inlineStr">
         <is>
           <t>시니어 입장: PENDING</t>
         </is>
       </c>
-      <c r="D132" s="25" t="inlineStr">
+      <c r="D133" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E132" s="25" t="inlineStr">
+      <c r="E133" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="133" ht="15" customHeight="1">
-      <c r="A133" s="26" t="inlineStr">
+    <row r="134" ht="15" customHeight="1">
+      <c r="A134" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position</t>
         </is>
       </c>
-      <c r="B133" s="26" t="inlineStr">
+      <c r="B134" s="26" t="inlineStr">
         <is>
           <t>AGREED</t>
         </is>
       </c>
-      <c r="C133" s="26" t="inlineStr">
+      <c r="C134" s="26" t="inlineStr">
         <is>
           <t>시니어 입장: AGREED</t>
         </is>
       </c>
-      <c r="D133" s="26" t="inlineStr">
+      <c r="D134" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E133" s="26" t="inlineStr">
+      <c r="E134" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="15" customHeight="1">
-      <c r="A134" s="25" t="inlineStr">
+    <row r="135" ht="15" customHeight="1">
+      <c r="A135" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position</t>
         </is>
       </c>
-      <c r="B134" s="25" t="inlineStr">
+      <c r="B135" s="25" t="inlineStr">
         <is>
           <t>DISAGREED</t>
         </is>
       </c>
-      <c r="C134" s="25" t="inlineStr">
+      <c r="C135" s="25" t="inlineStr">
         <is>
           <t>시니어 입장: DISAGREED</t>
         </is>
       </c>
-      <c r="D134" s="25" t="inlineStr">
+      <c r="D135" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E134" s="25" t="inlineStr">
+      <c r="E135" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="15" customHeight="1">
-      <c r="A135" s="26" t="inlineStr">
+    <row r="136" ht="15" customHeight="1">
+      <c r="A136" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position</t>
         </is>
       </c>
-      <c r="B135" s="26" t="inlineStr">
+      <c r="B136" s="26" t="inlineStr">
         <is>
           <t>UNREACHABLE</t>
         </is>
       </c>
-      <c r="C135" s="26" t="inlineStr">
+      <c r="C136" s="26" t="inlineStr">
         <is>
           <t>시니어 입장: UNREACHABLE</t>
         </is>
       </c>
-      <c r="D135" s="26" t="inlineStr">
+      <c r="D136" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.senior_position의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E135" s="26" t="inlineStr">
+      <c r="E136" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="15" customHeight="1">
-      <c r="A136" s="25" t="inlineStr">
+    <row r="137" ht="15" customHeight="1">
+      <c r="A137" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision</t>
         </is>
       </c>
-      <c r="B136" s="25" t="inlineStr">
+      <c r="B137" s="25" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="C136" s="25" t="inlineStr">
+      <c r="C137" s="25" t="inlineStr">
         <is>
           <t>PRIMARY 결정: PENDING</t>
         </is>
       </c>
-      <c r="D136" s="25" t="inlineStr">
+      <c r="D137" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E136" s="25" t="inlineStr">
+      <c r="E137" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="15" customHeight="1">
-      <c r="A137" s="26" t="inlineStr">
+    <row r="138" ht="15" customHeight="1">
+      <c r="A138" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision</t>
         </is>
       </c>
-      <c r="B137" s="26" t="inlineStr">
+      <c r="B138" s="26" t="inlineStr">
         <is>
           <t>CONFIRMED_EXISTING_VALUE</t>
         </is>
       </c>
-      <c r="C137" s="26" t="inlineStr">
+      <c r="C138" s="26" t="inlineStr">
         <is>
           <t>PRIMARY 결정: CONFIRMED_EXISTING_VALUE</t>
         </is>
       </c>
-      <c r="D137" s="26" t="inlineStr">
+      <c r="D138" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E137" s="26" t="inlineStr">
+      <c r="E138" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="138" ht="15" customHeight="1">
-      <c r="A138" s="25" t="inlineStr">
+    <row r="139" ht="15" customHeight="1">
+      <c r="A139" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision</t>
         </is>
       </c>
-      <c r="B138" s="25" t="inlineStr">
+      <c r="B139" s="25" t="inlineStr">
         <is>
           <t>CONFIRMED_PROPOSED_VALUE</t>
         </is>
       </c>
-      <c r="C138" s="25" t="inlineStr">
+      <c r="C139" s="25" t="inlineStr">
         <is>
           <t>PRIMARY 결정: CONFIRMED_PROPOSED_VALUE</t>
         </is>
       </c>
-      <c r="D138" s="25" t="inlineStr">
+      <c r="D139" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E138" s="25" t="inlineStr">
+      <c r="E139" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="15" customHeight="1">
-      <c r="A139" s="26" t="inlineStr">
+    <row r="140" ht="15" customHeight="1">
+      <c r="A140" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision</t>
         </is>
       </c>
-      <c r="B139" s="26" t="inlineStr">
+      <c r="B140" s="26" t="inlineStr">
         <is>
           <t>REVISED_VALUE</t>
         </is>
       </c>
-      <c r="C139" s="26" t="inlineStr">
+      <c r="C140" s="26" t="inlineStr">
         <is>
           <t>PRIMARY 결정: REVISED_VALUE</t>
         </is>
       </c>
-      <c r="D139" s="26" t="inlineStr">
+      <c r="D140" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E139" s="26" t="inlineStr">
+      <c r="E140" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="140" ht="15" customHeight="1">
-      <c r="A140" s="25" t="inlineStr">
+    <row r="141" ht="15" customHeight="1">
+      <c r="A141" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision</t>
         </is>
       </c>
-      <c r="B140" s="25" t="inlineStr">
+      <c r="B141" s="25" t="inlineStr">
         <is>
           <t>CANCELLED_CHANGE</t>
         </is>
       </c>
-      <c r="C140" s="25" t="inlineStr">
+      <c r="C141" s="25" t="inlineStr">
         <is>
           <t>PRIMARY 결정: CANCELLED_CHANGE</t>
         </is>
       </c>
-      <c r="D140" s="25" t="inlineStr">
+      <c r="D141" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.primary_guardian_decision의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E140" s="25" t="inlineStr">
+      <c r="E141" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="141" ht="15" customHeight="1">
-      <c r="A141" s="26" t="inlineStr">
+    <row r="142" ht="15" customHeight="1">
+      <c r="A142" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason</t>
         </is>
       </c>
-      <c r="B141" s="26" t="inlineStr">
+      <c r="B142" s="26" t="inlineStr">
         <is>
           <t>NO_RESPONSE</t>
         </is>
       </c>
-      <c r="C141" s="26" t="inlineStr">
+      <c r="C142" s="26" t="inlineStr">
         <is>
           <t>연락 불가 사유: NO_RESPONSE</t>
         </is>
       </c>
-      <c r="D141" s="26" t="inlineStr">
+      <c r="D142" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E141" s="26" t="inlineStr">
+      <c r="E142" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="142" ht="15" customHeight="1">
-      <c r="A142" s="25" t="inlineStr">
+    <row r="143" ht="15" customHeight="1">
+      <c r="A143" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason</t>
         </is>
       </c>
-      <c r="B142" s="25" t="inlineStr">
+      <c r="B143" s="25" t="inlineStr">
         <is>
           <t>PHONE_UNAVAILABLE</t>
         </is>
       </c>
-      <c r="C142" s="25" t="inlineStr">
+      <c r="C143" s="25" t="inlineStr">
         <is>
           <t>연락 불가 사유: PHONE_UNAVAILABLE</t>
         </is>
       </c>
-      <c r="D142" s="25" t="inlineStr">
+      <c r="D143" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E142" s="25" t="inlineStr">
+      <c r="E143" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="143" ht="15" customHeight="1">
-      <c r="A143" s="26" t="inlineStr">
+    <row r="144" ht="15" customHeight="1">
+      <c r="A144" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason</t>
         </is>
       </c>
-      <c r="B143" s="26" t="inlineStr">
+      <c r="B144" s="26" t="inlineStr">
         <is>
           <t>TEMPORARY_HEALTH_CONDITION</t>
         </is>
       </c>
-      <c r="C143" s="26" t="inlineStr">
+      <c r="C144" s="26" t="inlineStr">
         <is>
           <t>연락 불가 사유: TEMPORARY_HEALTH_CONDITION</t>
         </is>
       </c>
-      <c r="D143" s="26" t="inlineStr">
+      <c r="D144" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E143" s="26" t="inlineStr">
+      <c r="E144" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="144" ht="15" customHeight="1">
-      <c r="A144" s="25" t="inlineStr">
+    <row r="145" ht="15" customHeight="1">
+      <c r="A145" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason</t>
         </is>
       </c>
-      <c r="B144" s="25" t="inlineStr">
+      <c r="B145" s="25" t="inlineStr">
         <is>
           <t>COMMUNICATION_DIFFICULTY</t>
         </is>
       </c>
-      <c r="C144" s="25" t="inlineStr">
+      <c r="C145" s="25" t="inlineStr">
         <is>
           <t>연락 불가 사유: COMMUNICATION_DIFFICULTY</t>
         </is>
       </c>
-      <c r="D144" s="25" t="inlineStr">
+      <c r="D145" s="25" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E144" s="25" t="inlineStr">
+      <c r="E145" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="15" customHeight="1">
-      <c r="A145" s="26" t="inlineStr">
+    <row r="146" ht="15" customHeight="1">
+      <c r="A146" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason</t>
         </is>
       </c>
-      <c r="B145" s="26" t="inlineStr">
+      <c r="B146" s="26" t="inlineStr">
         <is>
           <t>OTHER</t>
         </is>
       </c>
-      <c r="C145" s="26" t="inlineStr">
+      <c r="C146" s="26" t="inlineStr">
         <is>
           <t>연락 불가 사유: OTHER</t>
         </is>
       </c>
-      <c r="D145" s="26" t="inlineStr">
+      <c r="D146" s="26" t="inlineStr">
         <is>
           <t>fact_candidate.unreachable_reason의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E145" s="26" t="inlineStr">
+      <c r="E146" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="146" ht="15" customHeight="1">
-      <c r="A146" s="25" t="inlineStr">
+    <row r="147" ht="15" customHeight="1">
+      <c r="A147" s="25" t="inlineStr">
         <is>
           <t>memory.memory_type</t>
         </is>
       </c>
-      <c r="B146" s="25" t="inlineStr">
+      <c r="B147" s="25" t="inlineStr">
         <is>
           <t>PERSONAL_RELATIONSHIP</t>
         </is>
       </c>
-      <c r="C146" s="25" t="inlineStr">
+      <c r="C147" s="25" t="inlineStr">
         <is>
           <t>장기 기억 유형: PERSONAL_RELATIONSHIP</t>
         </is>
       </c>
-      <c r="D146" s="25" t="inlineStr">
+      <c r="D147" s="25" t="inlineStr">
         <is>
           <t>memory.memory_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E146" s="25" t="inlineStr">
+      <c r="E147" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="147" ht="15" customHeight="1">
-      <c r="A147" s="26" t="inlineStr">
+    <row r="148" ht="15" customHeight="1">
+      <c r="A148" s="26" t="inlineStr">
         <is>
           <t>memory.memory_type</t>
         </is>
       </c>
-      <c r="B147" s="26" t="inlineStr">
+      <c r="B148" s="26" t="inlineStr">
         <is>
           <t>PREFERENCE</t>
         </is>
       </c>
-      <c r="C147" s="26" t="inlineStr">
+      <c r="C148" s="26" t="inlineStr">
         <is>
           <t>장기 기억 유형: PREFERENCE</t>
         </is>
       </c>
-      <c r="D147" s="26" t="inlineStr">
+      <c r="D148" s="26" t="inlineStr">
         <is>
           <t>memory.memory_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E147" s="26" t="inlineStr">
+      <c r="E148" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="148" ht="15" customHeight="1">
-      <c r="A148" s="25" t="inlineStr">
+    <row r="149" ht="15" customHeight="1">
+      <c r="A149" s="25" t="inlineStr">
         <is>
           <t>memory.memory_type</t>
         </is>
       </c>
-      <c r="B148" s="25" t="inlineStr">
+      <c r="B149" s="25" t="inlineStr">
         <is>
           <t>HOBBY</t>
         </is>
       </c>
-      <c r="C148" s="25" t="inlineStr">
+      <c r="C149" s="25" t="inlineStr">
         <is>
           <t>장기 기억 유형: HOBBY</t>
         </is>
       </c>
-      <c r="D148" s="25" t="inlineStr">
+      <c r="D149" s="25" t="inlineStr">
         <is>
           <t>memory.memory_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E148" s="25" t="inlineStr">
+      <c r="E149" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="15" customHeight="1">
-      <c r="A149" s="26" t="inlineStr">
+    <row r="150" ht="15" customHeight="1">
+      <c r="A150" s="26" t="inlineStr">
         <is>
           <t>memory.memory_type</t>
         </is>
       </c>
-      <c r="B149" s="26" t="inlineStr">
+      <c r="B150" s="26" t="inlineStr">
         <is>
           <t>DAILY_ROUTINE</t>
         </is>
       </c>
-      <c r="C149" s="26" t="inlineStr">
+      <c r="C150" s="26" t="inlineStr">
         <is>
           <t>장기 기억 유형: DAILY_ROUTINE</t>
         </is>
       </c>
-      <c r="D149" s="26" t="inlineStr">
+      <c r="D150" s="26" t="inlineStr">
         <is>
           <t>memory.memory_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E149" s="26" t="inlineStr">
+      <c r="E150" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="150" ht="15" customHeight="1">
-      <c r="A150" s="25" t="inlineStr">
+    <row r="151" ht="15" customHeight="1">
+      <c r="A151" s="25" t="inlineStr">
         <is>
           <t>memory.memory_type</t>
         </is>
       </c>
-      <c r="B150" s="25" t="inlineStr">
+      <c r="B151" s="25" t="inlineStr">
         <is>
           <t>LIFE_EVENT</t>
         </is>
       </c>
-      <c r="C150" s="25" t="inlineStr">
+      <c r="C151" s="25" t="inlineStr">
         <is>
           <t>장기 기억 유형: LIFE_EVENT</t>
         </is>
       </c>
-      <c r="D150" s="25" t="inlineStr">
+      <c r="D151" s="25" t="inlineStr">
         <is>
           <t>memory.memory_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E150" s="25" t="inlineStr">
+      <c r="E151" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="151" ht="15" customHeight="1">
-      <c r="A151" s="26" t="inlineStr">
+    <row r="152" ht="15" customHeight="1">
+      <c r="A152" s="26" t="inlineStr">
         <is>
           <t>memory.memory_type</t>
         </is>
       </c>
-      <c r="B151" s="26" t="inlineStr">
+      <c r="B152" s="26" t="inlineStr">
         <is>
           <t>FAMILY_MEMORY</t>
         </is>
       </c>
-      <c r="C151" s="26" t="inlineStr">
+      <c r="C152" s="26" t="inlineStr">
         <is>
           <t>장기 기억 유형: FAMILY_MEMORY</t>
         </is>
       </c>
-      <c r="D151" s="26" t="inlineStr">
+      <c r="D152" s="26" t="inlineStr">
         <is>
           <t>memory.memory_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E151" s="26" t="inlineStr">
+      <c r="E152" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="152" ht="15" customHeight="1">
-      <c r="A152" s="25" t="inlineStr">
+    <row r="153" ht="15" customHeight="1">
+      <c r="A153" s="25" t="inlineStr">
         <is>
           <t>memory.memory_type</t>
         </is>
       </c>
-      <c r="B152" s="25" t="inlineStr">
+      <c r="B153" s="25" t="inlineStr">
         <is>
           <t>EMOTIONAL_EVENT</t>
         </is>
       </c>
-      <c r="C152" s="25" t="inlineStr">
+      <c r="C153" s="25" t="inlineStr">
         <is>
           <t>장기 기억 유형: EMOTIONAL_EVENT</t>
         </is>
       </c>
-      <c r="D152" s="25" t="inlineStr">
+      <c r="D153" s="25" t="inlineStr">
         <is>
           <t>memory.memory_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E152" s="25" t="inlineStr">
+      <c r="E153" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="153" ht="15" customHeight="1">
-      <c r="A153" s="26" t="inlineStr">
+    <row r="154" ht="15" customHeight="1">
+      <c r="A154" s="26" t="inlineStr">
         <is>
           <t>memory.memory_type</t>
         </is>
       </c>
-      <c r="B153" s="26" t="inlineStr">
+      <c r="B154" s="26" t="inlineStr">
         <is>
           <t>OTHER</t>
         </is>
       </c>
-      <c r="C153" s="26" t="inlineStr">
+      <c r="C154" s="26" t="inlineStr">
         <is>
           <t>장기 기억 유형: OTHER</t>
         </is>
       </c>
-      <c r="D153" s="26" t="inlineStr">
+      <c r="D154" s="26" t="inlineStr">
         <is>
           <t>memory.memory_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E153" s="26" t="inlineStr">
+      <c r="E154" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="154" ht="15" customHeight="1">
-      <c r="A154" s="25" t="inlineStr">
+    <row r="155" ht="15" customHeight="1">
+      <c r="A155" s="25" t="inlineStr">
         <is>
           <t>memory.lifecycle_status</t>
         </is>
       </c>
-      <c r="B154" s="25" t="inlineStr">
+      <c r="B155" s="25" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="C154" s="25" t="inlineStr">
+      <c r="C155" s="25" t="inlineStr">
         <is>
           <t>기억 수명: ACTIVE</t>
         </is>
       </c>
-      <c r="D154" s="25" t="inlineStr">
+      <c r="D155" s="25" t="inlineStr">
         <is>
           <t>memory.lifecycle_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E154" s="25" t="inlineStr">
+      <c r="E155" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="155" ht="15" customHeight="1">
-      <c r="A155" s="26" t="inlineStr">
+    <row r="156" ht="15" customHeight="1">
+      <c r="A156" s="26" t="inlineStr">
         <is>
           <t>memory.lifecycle_status</t>
         </is>
       </c>
-      <c r="B155" s="26" t="inlineStr">
+      <c r="B156" s="26" t="inlineStr">
         <is>
           <t>DISPUTED</t>
         </is>
       </c>
-      <c r="C155" s="26" t="inlineStr">
+      <c r="C156" s="26" t="inlineStr">
         <is>
           <t>기억 수명: DISPUTED</t>
         </is>
       </c>
-      <c r="D155" s="26" t="inlineStr">
+      <c r="D156" s="26" t="inlineStr">
         <is>
           <t>memory.lifecycle_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E155" s="26" t="inlineStr">
+      <c r="E156" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="156" ht="15" customHeight="1">
-      <c r="A156" s="25" t="inlineStr">
+    <row r="157" ht="15" customHeight="1">
+      <c r="A157" s="25" t="inlineStr">
         <is>
           <t>memory.lifecycle_status</t>
         </is>
       </c>
-      <c r="B156" s="25" t="inlineStr">
+      <c r="B157" s="25" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
         </is>
       </c>
-      <c r="C156" s="25" t="inlineStr">
+      <c r="C157" s="25" t="inlineStr">
         <is>
           <t>기억 수명: SUPERSEDED</t>
         </is>
       </c>
-      <c r="D156" s="25" t="inlineStr">
+      <c r="D157" s="25" t="inlineStr">
         <is>
           <t>memory.lifecycle_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E156" s="25" t="inlineStr">
+      <c r="E157" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="157" ht="15" customHeight="1">
-      <c r="A157" s="26" t="inlineStr">
+    <row r="158" ht="15" customHeight="1">
+      <c r="A158" s="26" t="inlineStr">
         <is>
           <t>memory.lifecycle_status</t>
         </is>
       </c>
-      <c r="B157" s="26" t="inlineStr">
+      <c r="B158" s="26" t="inlineStr">
         <is>
           <t>EXPIRED</t>
         </is>
       </c>
-      <c r="C157" s="26" t="inlineStr">
+      <c r="C158" s="26" t="inlineStr">
         <is>
           <t>기억 수명: EXPIRED</t>
         </is>
       </c>
-      <c r="D157" s="26" t="inlineStr">
+      <c r="D158" s="26" t="inlineStr">
         <is>
           <t>memory.lifecycle_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E157" s="26" t="inlineStr">
+      <c r="E158" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="158" ht="15" customHeight="1">
-      <c r="A158" s="25" t="inlineStr">
+    <row r="159" ht="15" customHeight="1">
+      <c r="A159" s="25" t="inlineStr">
         <is>
           <t>memory.lifecycle_status</t>
         </is>
       </c>
-      <c r="B158" s="25" t="inlineStr">
+      <c r="B159" s="25" t="inlineStr">
         <is>
           <t>DELETED</t>
         </is>
       </c>
-      <c r="C158" s="25" t="inlineStr">
+      <c r="C159" s="25" t="inlineStr">
         <is>
           <t>기억 수명: DELETED</t>
         </is>
       </c>
-      <c r="D158" s="25" t="inlineStr">
+      <c r="D159" s="25" t="inlineStr">
         <is>
           <t>memory.lifecycle_status의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E158" s="25" t="inlineStr">
+      <c r="E159" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="159" ht="15" customHeight="1">
-      <c r="A159" s="26" t="inlineStr">
+    <row r="160" ht="15" customHeight="1">
+      <c r="A160" s="26" t="inlineStr">
         <is>
           <t>memory.visibility</t>
         </is>
       </c>
-      <c r="B159" s="26" t="inlineStr">
+      <c r="B160" s="26" t="inlineStr">
         <is>
           <t>PRIVATE</t>
         </is>
       </c>
-      <c r="C159" s="26" t="inlineStr">
+      <c r="C160" s="26" t="inlineStr">
         <is>
           <t>기억 공개 범위: PRIVATE</t>
         </is>
       </c>
-      <c r="D159" s="26" t="inlineStr">
+      <c r="D160" s="26" t="inlineStr">
         <is>
           <t>memory.visibility의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E159" s="26" t="inlineStr">
+      <c r="E160" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="160" ht="15" customHeight="1">
-      <c r="A160" s="25" t="inlineStr">
+    <row r="161" ht="15" customHeight="1">
+      <c r="A161" s="25" t="inlineStr">
         <is>
           <t>memory.visibility</t>
         </is>
       </c>
-      <c r="B160" s="25" t="inlineStr">
+      <c r="B161" s="25" t="inlineStr">
         <is>
           <t>SHARED_WITH_PRIMARY</t>
         </is>
       </c>
-      <c r="C160" s="25" t="inlineStr">
+      <c r="C161" s="25" t="inlineStr">
         <is>
           <t>기억 공개 범위: SHARED_WITH_PRIMARY</t>
         </is>
       </c>
-      <c r="D160" s="25" t="inlineStr">
+      <c r="D161" s="25" t="inlineStr">
         <is>
           <t>memory.visibility의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E160" s="25" t="inlineStr">
+      <c r="E161" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="161" ht="15" customHeight="1">
-      <c r="A161" s="26" t="inlineStr">
+    <row r="162" ht="15" customHeight="1">
+      <c r="A162" s="26" t="inlineStr">
         <is>
           <t>memory.visibility</t>
         </is>
       </c>
-      <c r="B161" s="26" t="inlineStr">
+      <c r="B162" s="26" t="inlineStr">
         <is>
           <t>SHARED_WITH_GUARDIANS</t>
         </is>
       </c>
-      <c r="C161" s="26" t="inlineStr">
+      <c r="C162" s="26" t="inlineStr">
         <is>
           <t>기억 공개 범위: SHARED_WITH_GUARDIANS</t>
         </is>
       </c>
-      <c r="D161" s="26" t="inlineStr">
+      <c r="D162" s="26" t="inlineStr">
         <is>
           <t>memory.visibility의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E161" s="26" t="inlineStr">
+      <c r="E162" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="162" ht="15" customHeight="1">
-      <c r="A162" s="25" t="inlineStr">
+    <row r="163" ht="15" customHeight="1">
+      <c r="A163" s="25" t="inlineStr">
         <is>
           <t>care_record.record_type</t>
         </is>
       </c>
-      <c r="B162" s="25" t="inlineStr">
+      <c r="B163" s="25" t="inlineStr">
         <is>
           <t>HEALTH_CONDITION</t>
         </is>
       </c>
-      <c r="C162" s="25" t="inlineStr">
+      <c r="C163" s="25" t="inlineStr">
         <is>
           <t>돌봄 기록 유형: HEALTH_CONDITION</t>
         </is>
       </c>
-      <c r="D162" s="25" t="inlineStr">
+      <c r="D163" s="25" t="inlineStr">
         <is>
           <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E162" s="25" t="inlineStr">
+      <c r="E163" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="163" ht="15" customHeight="1">
-      <c r="A163" s="26" t="inlineStr">
+    <row r="164" ht="15" customHeight="1">
+      <c r="A164" s="26" t="inlineStr">
         <is>
           <t>care_record.record_type</t>
         </is>
       </c>
-      <c r="B163" s="26" t="inlineStr">
+      <c r="B164" s="26" t="inlineStr">
         <is>
           <t>ALLERGY</t>
         </is>
       </c>
-      <c r="C163" s="26" t="inlineStr">
+      <c r="C164" s="26" t="inlineStr">
         <is>
           <t>돌봄 기록 유형: ALLERGY</t>
         </is>
       </c>
-      <c r="D163" s="26" t="inlineStr">
+      <c r="D164" s="26" t="inlineStr">
         <is>
           <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E163" s="26" t="inlineStr">
+      <c r="E164" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="164" ht="15" customHeight="1">
-      <c r="A164" s="25" t="inlineStr">
+    <row r="165" ht="15" customHeight="1">
+      <c r="A165" s="25" t="inlineStr">
         <is>
           <t>care_record.record_type</t>
         </is>
       </c>
-      <c r="B164" s="25" t="inlineStr">
+      <c r="B165" s="25" t="inlineStr">
         <is>
           <t>PHYSICAL_LIMITATION</t>
         </is>
       </c>
-      <c r="C164" s="25" t="inlineStr">
+      <c r="C165" s="25" t="inlineStr">
         <is>
           <t>돌봄 기록 유형: PHYSICAL_LIMITATION</t>
         </is>
       </c>
-      <c r="D164" s="25" t="inlineStr">
+      <c r="D165" s="25" t="inlineStr">
         <is>
           <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E164" s="25" t="inlineStr">
+      <c r="E165" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="165" ht="15" customHeight="1">
-      <c r="A165" s="26" t="inlineStr">
+    <row r="166" ht="15" customHeight="1">
+      <c r="A166" s="26" t="inlineStr">
         <is>
           <t>care_record.record_type</t>
         </is>
       </c>
-      <c r="B165" s="26" t="inlineStr">
+      <c r="B166" s="26" t="inlineStr">
         <is>
           <t>MEDICATION</t>
         </is>
       </c>
-      <c r="C165" s="26" t="inlineStr">
+      <c r="C166" s="26" t="inlineStr">
         <is>
           <t>돌봄 기록 유형: MEDICATION</t>
         </is>
       </c>
-      <c r="D165" s="26" t="inlineStr">
+      <c r="D166" s="26" t="inlineStr">
         <is>
           <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E165" s="26" t="inlineStr">
+      <c r="E166" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="166" ht="15" customHeight="1">
-      <c r="A166" s="25" t="inlineStr">
+    <row r="167" ht="15" customHeight="1">
+      <c r="A167" s="25" t="inlineStr">
         <is>
           <t>care_record.record_type</t>
         </is>
       </c>
-      <c r="B166" s="25" t="inlineStr">
+      <c r="B167" s="25" t="inlineStr">
         <is>
           <t>MEDICATION_SCHEDULE</t>
         </is>
       </c>
-      <c r="C166" s="25" t="inlineStr">
+      <c r="C167" s="25" t="inlineStr">
         <is>
           <t>돌봄 기록 유형: MEDICATION_SCHEDULE</t>
         </is>
       </c>
-      <c r="D166" s="25" t="inlineStr">
+      <c r="D167" s="25" t="inlineStr">
         <is>
           <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E166" s="25" t="inlineStr">
+      <c r="E167" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="167" ht="15" customHeight="1">
-      <c r="A167" s="26" t="inlineStr">
+    <row r="168" ht="15" customHeight="1">
+      <c r="A168" s="26" t="inlineStr">
         <is>
           <t>care_record.record_type</t>
         </is>
       </c>
-      <c r="B167" s="26" t="inlineStr">
+      <c r="B168" s="26" t="inlineStr">
         <is>
           <t>MEDICATION_REMINDER</t>
         </is>
       </c>
-      <c r="C167" s="26" t="inlineStr">
+      <c r="C168" s="26" t="inlineStr">
         <is>
           <t>돌봄 기록 유형: MEDICATION_REMINDER</t>
         </is>
       </c>
-      <c r="D167" s="26" t="inlineStr">
+      <c r="D168" s="26" t="inlineStr">
         <is>
           <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E167" s="26" t="inlineStr">
+      <c r="E168" s="26" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="168" ht="15" customHeight="1">
-      <c r="A168" s="25" t="inlineStr">
+    <row r="169" ht="15" customHeight="1">
+      <c r="A169" s="25" t="inlineStr">
         <is>
           <t>care_record.record_type</t>
         </is>
       </c>
-      <c r="B168" s="25" t="inlineStr">
+      <c r="B169" s="25" t="inlineStr">
         <is>
           <t>MEDICATION_TAKEN</t>
         </is>
       </c>
-      <c r="C168" s="25" t="inlineStr">
+      <c r="C169" s="25" t="inlineStr">
         <is>
           <t>돌봄 기록 유형: MEDICATION_TAKEN</t>
         </is>
       </c>
-      <c r="D168" s="25" t="inlineStr">
+      <c r="D169" s="25" t="inlineStr">
         <is>
           <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E168" s="25" t="inlineStr">
+      <c r="E169" s="25" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
-    <row r="169" ht="15" customHeight="1">
-      <c r="A169" s="28" t="inlineStr">
+    <row r="170" ht="15" customHeight="1">
+      <c r="A170" s="28" t="inlineStr">
         <is>
           <t>care_record.record_type</t>
         </is>
       </c>
-      <c r="B169" s="28" t="inlineStr">
+      <c r="B170" s="28" t="inlineStr">
         <is>
           <t>APPOINTMENT</t>
         </is>
       </c>
-      <c r="C169" s="28" t="inlineStr">
+      <c r="C170" s="28" t="inlineStr">
         <is>
           <t>돌봄 기록 유형: APPOINTMENT</t>
         </is>
       </c>
-      <c r="D169" s="28" t="inlineStr">
+      <c r="D170" s="28" t="inlineStr">
         <is>
           <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
-      <c r="E169" s="28" t="inlineStr">
-        <is>
-          <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
-        </is>
-      </c>
-    </row>
-    <row r="170" ht="15" customHeight="1">
-      <c r="A170" s="32" t="inlineStr">
-        <is>
-          <t>care_record.record_type</t>
-        </is>
-      </c>
-      <c r="B170" s="32" t="inlineStr">
-        <is>
-          <t>PERSONAL_SCHEDULE</t>
-        </is>
-      </c>
-      <c r="C170" s="32" t="inlineStr">
-        <is>
-          <t>돌봄 기록 유형: PERSONAL_SCHEDULE</t>
-        </is>
-      </c>
-      <c r="D170" s="32" t="inlineStr">
-        <is>
-          <t>care_record.record_type의 상태·분기 판단</t>
-        </is>
-      </c>
-      <c r="E170" s="32" t="inlineStr">
+      <c r="E170" s="28" t="inlineStr">
         <is>
           <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
@@ -23481,12 +23501,12 @@
       </c>
       <c r="B171" s="32" t="inlineStr">
         <is>
-          <t>HEALTH_OBSERVATION</t>
+          <t>PERSONAL_SCHEDULE</t>
         </is>
       </c>
       <c r="C171" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 유형: HEALTH_OBSERVATION</t>
+          <t>돌봄 기록 유형: PERSONAL_SCHEDULE</t>
         </is>
       </c>
       <c r="D171" s="32" t="inlineStr">
@@ -23508,12 +23528,12 @@
       </c>
       <c r="B172" s="32" t="inlineStr">
         <is>
-          <t>REST_OBSERVATION</t>
+          <t>HEALTH_OBSERVATION</t>
         </is>
       </c>
       <c r="C172" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 유형: REST_OBSERVATION</t>
+          <t>돌봄 기록 유형: HEALTH_OBSERVATION</t>
         </is>
       </c>
       <c r="D172" s="32" t="inlineStr">
@@ -23535,12 +23555,12 @@
       </c>
       <c r="B173" s="32" t="inlineStr">
         <is>
-          <t>ENVIRONMENT_OBSERVATION</t>
+          <t>REST_OBSERVATION</t>
         </is>
       </c>
       <c r="C173" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 유형: ENVIRONMENT_OBSERVATION</t>
+          <t>돌봄 기록 유형: REST_OBSERVATION</t>
         </is>
       </c>
       <c r="D173" s="32" t="inlineStr">
@@ -23562,12 +23582,12 @@
       </c>
       <c r="B174" s="32" t="inlineStr">
         <is>
-          <t>COGNITIVE_ASSESSMENT</t>
+          <t>ENVIRONMENT_OBSERVATION</t>
         </is>
       </c>
       <c r="C174" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 유형: COGNITIVE_ASSESSMENT</t>
+          <t>돌봄 기록 유형: ENVIRONMENT_OBSERVATION</t>
         </is>
       </c>
       <c r="D174" s="32" t="inlineStr">
@@ -23589,12 +23609,12 @@
       </c>
       <c r="B175" s="32" t="inlineStr">
         <is>
-          <t>GUARDIAN_NOTIFICATION</t>
+          <t>COGNITIVE_ASSESSMENT</t>
         </is>
       </c>
       <c r="C175" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 유형: GUARDIAN_NOTIFICATION</t>
+          <t>돌봄 기록 유형: COGNITIVE_ASSESSMENT</t>
         </is>
       </c>
       <c r="D175" s="32" t="inlineStr">
@@ -23611,22 +23631,22 @@
     <row r="176" ht="15" customHeight="1">
       <c r="A176" s="32" t="inlineStr">
         <is>
-          <t>care_record.status</t>
+          <t>care_record.record_type</t>
         </is>
       </c>
       <c r="B176" s="32" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>GUARDIAN_NOTIFICATION</t>
         </is>
       </c>
       <c r="C176" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 상태: ACTIVE</t>
+          <t>돌봄 기록 유형: GUARDIAN_NOTIFICATION</t>
         </is>
       </c>
       <c r="D176" s="32" t="inlineStr">
         <is>
-          <t>care_record.status의 상태·분기 판단</t>
+          <t>care_record.record_type의 상태·분기 판단</t>
         </is>
       </c>
       <c r="E176" s="32" t="inlineStr">
@@ -23643,12 +23663,12 @@
       </c>
       <c r="B177" s="32" t="inlineStr">
         <is>
-          <t>COMPLETED</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="C177" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 상태: COMPLETED</t>
+          <t>돌봄 기록 상태: ACTIVE</t>
         </is>
       </c>
       <c r="D177" s="32" t="inlineStr">
@@ -23670,12 +23690,12 @@
       </c>
       <c r="B178" s="32" t="inlineStr">
         <is>
-          <t>CANCELLED</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="C178" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 상태: CANCELLED</t>
+          <t>돌봄 기록 상태: COMPLETED</t>
         </is>
       </c>
       <c r="D178" s="32" t="inlineStr">
@@ -23697,12 +23717,12 @@
       </c>
       <c r="B179" s="32" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>CANCELLED</t>
         </is>
       </c>
       <c r="C179" s="32" t="inlineStr">
         <is>
-          <t>돌봄 기록 상태: SUPERSEDED</t>
+          <t>돌봄 기록 상태: CANCELLED</t>
         </is>
       </c>
       <c r="D179" s="32" t="inlineStr">
@@ -23719,22 +23739,22 @@
     <row r="180" ht="15" customHeight="1">
       <c r="A180" s="32" t="inlineStr">
         <is>
-          <t>care_record.recurrence.frequency</t>
+          <t>care_record.status</t>
         </is>
       </c>
       <c r="B180" s="32" t="inlineStr">
         <is>
-          <t>DAILY</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="C180" s="32" t="inlineStr">
         <is>
-          <t>반복 주기: DAILY</t>
+          <t>돌봄 기록 상태: SUPERSEDED</t>
         </is>
       </c>
       <c r="D180" s="32" t="inlineStr">
         <is>
-          <t>care_record.recurrence.frequency의 상태·분기 판단</t>
+          <t>care_record.status의 상태·분기 판단</t>
         </is>
       </c>
       <c r="E180" s="32" t="inlineStr">
@@ -23751,12 +23771,12 @@
       </c>
       <c r="B181" s="32" t="inlineStr">
         <is>
-          <t>WEEKLY</t>
+          <t>DAILY</t>
         </is>
       </c>
       <c r="C181" s="32" t="inlineStr">
         <is>
-          <t>반복 주기: WEEKLY</t>
+          <t>반복 주기: DAILY</t>
         </is>
       </c>
       <c r="D181" s="32" t="inlineStr">
@@ -23773,54 +23793,54 @@
     <row r="182" ht="15" customHeight="1">
       <c r="A182" s="32" t="inlineStr">
         <is>
-          <t>scenario.scenario_type</t>
+          <t>care_record.recurrence.frequency</t>
         </is>
       </c>
       <c r="B182" s="32" t="inlineStr">
         <is>
-          <t>WALK</t>
+          <t>WEEKLY</t>
         </is>
       </c>
       <c r="C182" s="32" t="inlineStr">
         <is>
-          <t>시나리오 유형: 산책</t>
+          <t>반복 주기: WEEKLY</t>
         </is>
       </c>
       <c r="D182" s="32" t="inlineStr">
         <is>
-          <t>scenario.scenario_type의 상태·분기 판단</t>
+          <t>care_record.recurrence.frequency의 상태·분기 판단</t>
         </is>
       </c>
       <c r="E182" s="32" t="inlineStr">
         <is>
-          <t>FOLLOW 제어만 관리하고 tracking은 Robot 책임</t>
+          <t>정의되지 않은 값을 성공으로 처리하지 않음</t>
         </is>
       </c>
     </row>
     <row r="183" ht="15" customHeight="1">
       <c r="A183" s="32" t="inlineStr">
         <is>
-          <t>scenario.final_status</t>
+          <t>scenario.scenario_type</t>
         </is>
       </c>
       <c r="B183" s="32" t="inlineStr">
         <is>
-          <t>STARTING_FOLLOW</t>
+          <t>WALK</t>
         </is>
       </c>
       <c r="C183" s="32" t="inlineStr">
         <is>
-          <t>FOLLOW_START 결과 대기</t>
+          <t>시나리오 유형: 산책</t>
         </is>
       </c>
       <c r="D183" s="32" t="inlineStr">
         <is>
-          <t>WALK 시작 명령 발행 뒤 사용</t>
+          <t>scenario.scenario_type의 상태·분기 판단</t>
         </is>
       </c>
       <c r="E183" s="32" t="inlineStr">
         <is>
-          <t>늦은 STARTED가 STOPPING을 되돌리지 않음</t>
+          <t>FOLLOW 제어만 관리하고 tracking은 Robot 책임</t>
         </is>
       </c>
     </row>
@@ -23832,22 +23852,22 @@
       </c>
       <c r="B184" s="32" t="inlineStr">
         <is>
-          <t>FOLLOWING</t>
+          <t>STARTING_FOLLOW</t>
         </is>
       </c>
       <c r="C184" s="32" t="inlineStr">
         <is>
-          <t>Robot 추종 진행 중</t>
+          <t>FOLLOW_START 결과 대기</t>
         </is>
       </c>
       <c r="D184" s="32" t="inlineStr">
         <is>
-          <t>유효한 STARTED·UNCHANGED 뒤 사용</t>
+          <t>WALK 시작 명령 발행 뒤 사용</t>
         </is>
       </c>
       <c r="E184" s="32" t="inlineStr">
         <is>
-          <t>공용 20분 watchdog에서 제외</t>
+          <t>늦은 STARTED가 STOPPING을 되돌리지 않음</t>
         </is>
       </c>
     </row>
@@ -23859,49 +23879,49 @@
       </c>
       <c r="B185" s="32" t="inlineStr">
         <is>
-          <t>STOPPING_FOLLOW</t>
+          <t>FOLLOWING</t>
         </is>
       </c>
       <c r="C185" s="32" t="inlineStr">
         <is>
-          <t>FOLLOW_STOP 결과 대기</t>
+          <t>Robot 추종 진행 중</t>
         </is>
       </c>
       <c r="D185" s="32" t="inlineStr">
         <is>
-          <t>명시적 STOP 또는 안전 종료 시 사용</t>
+          <t>유효한 STARTED·UNCHANGED 뒤 사용</t>
         </is>
       </c>
       <c r="E185" s="32" t="inlineStr">
         <is>
-          <t>같은 STOP 요청은 새 command를 만들지 않음</t>
+          <t>공용 20분 watchdog에서 제외</t>
         </is>
       </c>
     </row>
     <row r="186" ht="15" customHeight="1">
       <c r="A186" s="32" t="inlineStr">
         <is>
-          <t>walk_request_receipt.ingress</t>
+          <t>scenario.final_status</t>
         </is>
       </c>
       <c r="B186" s="32" t="inlineStr">
         <is>
-          <t>MQTT</t>
+          <t>STOPPING_FOLLOW</t>
         </is>
       </c>
       <c r="C186" s="32" t="inlineStr">
         <is>
-          <t>Voice/AI MQTT 유입</t>
+          <t>FOLLOW_STOP 결과 대기</t>
         </is>
       </c>
       <c r="D186" s="32" t="inlineStr">
         <is>
-          <t>request_id 멱등 범위를 정함</t>
+          <t>명시적 STOP 또는 안전 종료 시 사용</t>
         </is>
       </c>
       <c r="E186" s="32" t="inlineStr">
         <is>
-          <t>payload source와 구분</t>
+          <t>같은 STOP 요청은 새 command를 만들지 않음</t>
         </is>
       </c>
     </row>
@@ -23913,49 +23933,49 @@
       </c>
       <c r="B187" s="32" t="inlineStr">
         <is>
-          <t>GUARDIAN_REST</t>
+          <t>MQTT</t>
         </is>
       </c>
       <c r="C187" s="32" t="inlineStr">
         <is>
-          <t>Guardian REST 유입</t>
+          <t>Voice/AI MQTT 유입</t>
         </is>
       </c>
       <c r="D187" s="32" t="inlineStr">
         <is>
-          <t>App requestId 멱등 범위를 정함</t>
+          <t>request_id 멱등 범위를 정함</t>
         </is>
       </c>
       <c r="E187" s="32" t="inlineStr">
         <is>
-          <t>MQTT의 같은 문자열 ID와 충돌하지 않음</t>
+          <t>payload source와 구분</t>
         </is>
       </c>
     </row>
     <row r="188" ht="15" customHeight="1">
       <c r="A188" s="32" t="inlineStr">
         <is>
-          <t>walk_request_receipt.action</t>
+          <t>walk_request_receipt.ingress</t>
         </is>
       </c>
       <c r="B188" s="32" t="inlineStr">
         <is>
-          <t>START</t>
+          <t>GUARDIAN_REST</t>
         </is>
       </c>
       <c r="C188" s="32" t="inlineStr">
         <is>
-          <t>산책 시작 요청</t>
+          <t>Guardian REST 유입</t>
         </is>
       </c>
       <c r="D188" s="32" t="inlineStr">
         <is>
-          <t>새 WALK 입장 정책 실행</t>
+          <t>App requestId 멱등 범위를 정함</t>
         </is>
       </c>
       <c r="E188" s="32" t="inlineStr">
         <is>
-          <t>활성 시나리오를 선점하지 않음</t>
+          <t>MQTT의 같은 문자열 ID와 충돌하지 않음</t>
         </is>
       </c>
     </row>
@@ -23967,49 +23987,49 @@
       </c>
       <c r="B189" s="32" t="inlineStr">
         <is>
-          <t>STOP</t>
+          <t>START</t>
         </is>
       </c>
       <c r="C189" s="32" t="inlineStr">
         <is>
-          <t>산책 종료 요청</t>
+          <t>산책 시작 요청</t>
         </is>
       </c>
       <c r="D189" s="32" t="inlineStr">
         <is>
-          <t>같은 Robot의 활성 WALK를 잠금 조회</t>
+          <t>새 WALK 입장 정책 실행</t>
         </is>
       </c>
       <c r="E189" s="32" t="inlineStr">
         <is>
-          <t>새 Scenario를 만들지 않음</t>
+          <t>활성 시나리오를 선점하지 않음</t>
         </is>
       </c>
     </row>
     <row r="190" ht="15" customHeight="1">
       <c r="A190" s="32" t="inlineStr">
         <is>
-          <t>walk_request_receipt.source</t>
+          <t>walk_request_receipt.action</t>
         </is>
       </c>
       <c r="B190" s="32" t="inlineStr">
         <is>
-          <t>VOICE</t>
+          <t>STOP</t>
         </is>
       </c>
       <c r="C190" s="32" t="inlineStr">
         <is>
-          <t>음성 의도 판정 출처</t>
+          <t>산책 종료 요청</t>
         </is>
       </c>
       <c r="D190" s="32" t="inlineStr">
         <is>
-          <t>MQTT 요청 문맥 비교</t>
+          <t>같은 Robot의 활성 WALK를 잠금 조회</t>
         </is>
       </c>
       <c r="E190" s="32" t="inlineStr">
         <is>
-          <t>Backend가 대화 intent를 새로 만들지 않음</t>
+          <t>새 Scenario를 만들지 않음</t>
         </is>
       </c>
     </row>
@@ -24021,49 +24041,49 @@
       </c>
       <c r="B191" s="32" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>VOICE</t>
         </is>
       </c>
       <c r="C191" s="32" t="inlineStr">
         <is>
-          <t>Guardian App 출처</t>
+          <t>음성 의도 판정 출처</t>
         </is>
       </c>
       <c r="D191" s="32" t="inlineStr">
         <is>
-          <t>REST adapter가 서버에서 고정</t>
+          <t>MQTT 요청 문맥 비교</t>
         </is>
       </c>
       <c r="E191" s="32" t="inlineStr">
         <is>
-          <t>클라이언트가 다른 값으로 지정할 수 없음</t>
+          <t>Backend가 대화 intent를 새로 만들지 않음</t>
         </is>
       </c>
     </row>
     <row r="192" ht="15" customHeight="1">
       <c r="A192" s="32" t="inlineStr">
         <is>
-          <t>walk_request_receipt.disposition</t>
+          <t>walk_request_receipt.source</t>
         </is>
       </c>
       <c r="B192" s="32" t="inlineStr">
         <is>
-          <t>RECEIVED</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="C192" s="32" t="inlineStr">
         <is>
-          <t>처리 중 임시 결정</t>
+          <t>Guardian App 출처</t>
         </is>
       </c>
       <c r="D192" s="32" t="inlineStr">
         <is>
-          <t>영수증 생성 직후 사용</t>
+          <t>REST adapter가 서버에서 고정</t>
         </is>
       </c>
       <c r="E192" s="32" t="inlineStr">
         <is>
-          <t>최종 응답으로 해석하지 않음</t>
+          <t>클라이언트가 다른 값으로 지정할 수 없음</t>
         </is>
       </c>
     </row>
@@ -24075,22 +24095,22 @@
       </c>
       <c r="B193" s="32" t="inlineStr">
         <is>
-          <t>ACCEPTED</t>
+          <t>RECEIVED</t>
         </is>
       </c>
       <c r="C193" s="32" t="inlineStr">
         <is>
-          <t>새 FOLLOW 명령 수락</t>
+          <t>처리 중 임시 결정</t>
         </is>
       </c>
       <c r="D193" s="32" t="inlineStr">
         <is>
-          <t>START 또는 STOP 명령 발행 결정</t>
+          <t>영수증 생성 직후 사용</t>
         </is>
       </c>
       <c r="E193" s="32" t="inlineStr">
         <is>
-          <t>scenario_id·scenario_status 필수</t>
+          <t>최종 응답으로 해석하지 않음</t>
         </is>
       </c>
     </row>
@@ -24102,22 +24122,22 @@
       </c>
       <c r="B194" s="32" t="inlineStr">
         <is>
-          <t>NO_OP_ALREADY_STOPPING</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="C194" s="32" t="inlineStr">
         <is>
-          <t>이미 종료 명령 대기 중</t>
+          <t>새 FOLLOW 명령 수락</t>
         </is>
       </c>
       <c r="D194" s="32" t="inlineStr">
         <is>
-          <t>STOPPING 중 다른 STOP을 결정적으로 수락</t>
+          <t>START 또는 STOP 명령 발행 결정</t>
         </is>
       </c>
       <c r="E194" s="32" t="inlineStr">
         <is>
-          <t>기존 commandId를 다시 만들지 않음</t>
+          <t>scenario_id·scenario_status 필수</t>
         </is>
       </c>
     </row>
@@ -24129,22 +24149,22 @@
       </c>
       <c r="B195" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_NO_ACTIVE_WALK</t>
+          <t>NO_OP_ALREADY_STOPPING</t>
         </is>
       </c>
       <c r="C195" s="32" t="inlineStr">
         <is>
-          <t>종료할 활성 산책 없음</t>
+          <t>이미 종료 명령 대기 중</t>
         </is>
       </c>
       <c r="D195" s="32" t="inlineStr">
         <is>
-          <t>STOP without active 응답</t>
+          <t>STOPPING 중 다른 STOP을 결정적으로 수락</t>
         </is>
       </c>
       <c r="E195" s="32" t="inlineStr">
         <is>
-          <t>나중에 생긴 산책을 같은 ID로 멈추지 않음</t>
+          <t>기존 commandId를 다시 만들지 않음</t>
         </is>
       </c>
     </row>
@@ -24156,22 +24176,22 @@
       </c>
       <c r="B196" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_UNKNOWN_ROBOT</t>
+          <t>REJECTED_NO_ACTIVE_WALK</t>
         </is>
       </c>
       <c r="C196" s="32" t="inlineStr">
         <is>
-          <t>미등록 Robot</t>
+          <t>종료할 활성 산책 없음</t>
         </is>
       </c>
       <c r="D196" s="32" t="inlineStr">
         <is>
-          <t>deviceId 권위 조회 실패</t>
+          <t>STOP without active 응답</t>
         </is>
       </c>
       <c r="E196" s="32" t="inlineStr">
         <is>
-          <t>명령 미발행</t>
+          <t>나중에 생긴 산책을 같은 ID로 멈추지 않음</t>
         </is>
       </c>
     </row>
@@ -24183,22 +24203,22 @@
       </c>
       <c r="B197" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_INACTIVE_ROBOT</t>
+          <t>REJECTED_UNKNOWN_ROBOT</t>
         </is>
       </c>
       <c r="C197" s="32" t="inlineStr">
         <is>
-          <t>비활성 Robot</t>
+          <t>미등록 Robot</t>
         </is>
       </c>
       <c r="D197" s="32" t="inlineStr">
         <is>
-          <t>START 입장 정책</t>
+          <t>deviceId 권위 조회 실패</t>
         </is>
       </c>
       <c r="E197" s="32" t="inlineStr">
         <is>
-          <t>STOP 안전 시도에는 적용하지 않음</t>
+          <t>명령 미발행</t>
         </is>
       </c>
     </row>
@@ -24210,22 +24230,22 @@
       </c>
       <c r="B198" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_UNASSIGNED_ROBOT</t>
+          <t>REJECTED_INACTIVE_ROBOT</t>
         </is>
       </c>
       <c r="C198" s="32" t="inlineStr">
         <is>
-          <t>시니어 미배정 Robot</t>
+          <t>비활성 Robot</t>
         </is>
       </c>
       <c r="D198" s="32" t="inlineStr">
         <is>
-          <t>START 대상 검증</t>
+          <t>START 입장 정책</t>
         </is>
       </c>
       <c r="E198" s="32" t="inlineStr">
         <is>
-          <t>어르신 잠금 없이 시작하지 않음</t>
+          <t>STOP 안전 시도에는 적용하지 않음</t>
         </is>
       </c>
     </row>
@@ -24237,22 +24257,22 @@
       </c>
       <c r="B199" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_SAFE_STOP</t>
+          <t>REJECTED_UNASSIGNED_ROBOT</t>
         </is>
       </c>
       <c r="C199" s="32" t="inlineStr">
         <is>
-          <t>SAFE_STOP Robot</t>
+          <t>시니어 미배정 Robot</t>
         </is>
       </c>
       <c r="D199" s="32" t="inlineStr">
         <is>
-          <t>START 안전 정책</t>
+          <t>START 대상 검증</t>
         </is>
       </c>
       <c r="E199" s="32" t="inlineStr">
         <is>
-          <t>안전 정지 상태에서 추종을 시작하지 않음</t>
+          <t>어르신 잠금 없이 시작하지 않음</t>
         </is>
       </c>
     </row>
@@ -24264,22 +24284,22 @@
       </c>
       <c r="B200" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_REST_GUARD</t>
+          <t>REJECTED_SAFE_STOP</t>
         </is>
       </c>
       <c r="C200" s="32" t="inlineStr">
         <is>
-          <t>REST_GUARD Robot</t>
+          <t>SAFE_STOP Robot</t>
         </is>
       </c>
       <c r="D200" s="32" t="inlineStr">
         <is>
-          <t>START 휴식 보호 정책</t>
+          <t>START 안전 정책</t>
         </is>
       </c>
       <c r="E200" s="32" t="inlineStr">
         <is>
-          <t>휴식 상태를 산책이 선점하지 않음</t>
+          <t>안전 정지 상태에서 추종을 시작하지 않음</t>
         </is>
       </c>
     </row>
@@ -24291,22 +24311,22 @@
       </c>
       <c r="B201" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_ACTIVE_SCENARIO</t>
+          <t>REJECTED_REST_GUARD</t>
         </is>
       </c>
       <c r="C201" s="32" t="inlineStr">
         <is>
-          <t>다른 활성 시나리오 존재</t>
+          <t>REST_GUARD Robot</t>
         </is>
       </c>
       <c r="D201" s="32" t="inlineStr">
         <is>
-          <t>시니어 단위 시작 직렬화</t>
+          <t>START 휴식 보호 정책</t>
         </is>
       </c>
       <c r="E201" s="32" t="inlineStr">
         <is>
-          <t>기존 흐름을 취소하지 않음</t>
+          <t>휴식 상태를 산책이 선점하지 않음</t>
         </is>
       </c>
     </row>
@@ -24318,22 +24338,22 @@
       </c>
       <c r="B202" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_BUSY_MODE</t>
+          <t>REJECTED_ACTIVE_SCENARIO</t>
         </is>
       </c>
       <c r="C202" s="32" t="inlineStr">
         <is>
-          <t>지원하지 않는 활성 Robot mode</t>
+          <t>다른 활성 시나리오 존재</t>
         </is>
       </c>
       <c r="D202" s="32" t="inlineStr">
         <is>
-          <t>START mode 검사</t>
+          <t>시니어 단위 시작 직렬화</t>
         </is>
       </c>
       <c r="E202" s="32" t="inlineStr">
         <is>
-          <t>IDLE에서만 산책 시작</t>
+          <t>기존 흐름을 취소하지 않음</t>
         </is>
       </c>
     </row>
@@ -24345,22 +24365,22 @@
       </c>
       <c r="B203" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_REQUEST_ID_REUSED</t>
+          <t>REJECTED_BUSY_MODE</t>
         </is>
       </c>
       <c r="C203" s="32" t="inlineStr">
         <is>
-          <t>요청 ID 문맥 불일치</t>
+          <t>지원하지 않는 활성 Robot mode</t>
         </is>
       </c>
       <c r="D203" s="32" t="inlineStr">
         <is>
-          <t>같은 키의 robot/action/source 비교</t>
+          <t>START mode 검사</t>
         </is>
       </c>
       <c r="E203" s="32" t="inlineStr">
         <is>
-          <t>기존 결정을 덮어쓰지 않음</t>
+          <t>IDLE에서만 산책 시작</t>
         </is>
       </c>
     </row>
@@ -24372,49 +24392,49 @@
       </c>
       <c r="B204" s="32" t="inlineStr">
         <is>
-          <t>REJECTED_MQTT_UNAVAILABLE</t>
+          <t>REJECTED_REQUEST_ID_REUSED</t>
         </is>
       </c>
       <c r="C204" s="32" t="inlineStr">
         <is>
-          <t>명령 gateway 비활성</t>
+          <t>요청 ID 문맥 불일치</t>
         </is>
       </c>
       <c r="D204" s="32" t="inlineStr">
         <is>
-          <t>REST 문서 profile·운영 장애 응답</t>
+          <t>같은 키의 robot/action/source 비교</t>
         </is>
       </c>
       <c r="E204" s="32" t="inlineStr">
         <is>
-          <t>영수증을 확정하지 않아 재시도 가능</t>
+          <t>기존 결정을 덮어쓰지 않음</t>
         </is>
       </c>
     </row>
     <row r="205" ht="15" customHeight="1">
       <c r="A205" s="32" t="inlineStr">
         <is>
-          <t>scenario.last_follow_result_code</t>
+          <t>walk_request_receipt.disposition</t>
         </is>
       </c>
       <c r="B205" s="32" t="inlineStr">
         <is>
-          <t>STARTED</t>
+          <t>REJECTED_MQTT_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C205" s="32" t="inlineStr">
         <is>
-          <t>추종 시작 확인</t>
+          <t>명령 gateway 비활성</t>
         </is>
       </c>
       <c r="D205" s="32" t="inlineStr">
         <is>
-          <t>FOLLOW_START 성공 결과</t>
+          <t>REST 문서 profile·운영 장애 응답</t>
         </is>
       </c>
       <c r="E205" s="32" t="inlineStr">
         <is>
-          <t>START commandId와 함께 검증</t>
+          <t>영수증을 확정하지 않아 재시도 가능</t>
         </is>
       </c>
     </row>
@@ -24426,22 +24446,22 @@
       </c>
       <c r="B206" s="32" t="inlineStr">
         <is>
-          <t>STOPPED</t>
+          <t>STARTED</t>
         </is>
       </c>
       <c r="C206" s="32" t="inlineStr">
         <is>
-          <t>추종 종료 확인</t>
+          <t>추종 시작 확인</t>
         </is>
       </c>
       <c r="D206" s="32" t="inlineStr">
         <is>
-          <t>명시적 STOP 또는 Robot 자체 종료</t>
+          <t>FOLLOW_START 성공 결과</t>
         </is>
       </c>
       <c r="E206" s="32" t="inlineStr">
         <is>
-          <t>어느 commandId인지 함께 보존</t>
+          <t>START commandId와 함께 검증</t>
         </is>
       </c>
     </row>
@@ -24453,49 +24473,49 @@
       </c>
       <c r="B207" s="32" t="inlineStr">
         <is>
-          <t>UNCHANGED</t>
+          <t>STOPPED</t>
         </is>
       </c>
       <c r="C207" s="32" t="inlineStr">
         <is>
-          <t>이미 원하는 추종 상태 또는 Backend synthetic timeout 기록 코드</t>
+          <t>추종 종료 확인</t>
         </is>
       </c>
       <c r="D207" s="32" t="inlineStr">
         <is>
-          <t>Robot 멱등 성공 결과 또는 timeout- eventId의 Backend 안전 종료</t>
+          <t>명시적 STOP 또는 Robot 자체 종료</t>
         </is>
       </c>
       <c r="E207" s="32" t="inlineStr">
         <is>
-          <t>synthetic timeout은 Robot 성공 증거가 아니며 eventId·reasonCode와 함께 판별</t>
+          <t>어느 commandId인지 함께 보존</t>
         </is>
       </c>
     </row>
     <row r="208" ht="15" customHeight="1">
       <c r="A208" s="32" t="inlineStr">
         <is>
-          <t>scenario.last_follow_reason_code</t>
+          <t>scenario.last_follow_result_code</t>
         </is>
       </c>
       <c r="B208" s="32" t="inlineStr">
         <is>
-          <t>PERSON_LOST</t>
+          <t>UNCHANGED</t>
         </is>
       </c>
       <c r="C208" s="32" t="inlineStr">
         <is>
-          <t>추종 대상 놓침</t>
+          <t>이미 원하는 추종 상태 또는 Backend synthetic timeout 기록 코드</t>
         </is>
       </c>
       <c r="D208" s="32" t="inlineStr">
         <is>
-          <t>실패 FOLLOW_RESULT</t>
+          <t>Robot 멱등 성공 결과 또는 timeout- eventId의 Backend 안전 종료</t>
         </is>
       </c>
       <c r="E208" s="32" t="inlineStr">
         <is>
-          <t>고빈도 tracking 정보는 저장하지 않음</t>
+          <t>synthetic timeout은 Robot 성공 증거가 아니며 eventId·reasonCode와 함께 판별</t>
         </is>
       </c>
     </row>
@@ -24507,22 +24527,22 @@
       </c>
       <c r="B209" s="32" t="inlineStr">
         <is>
-          <t>COMMAND_EXPIRED</t>
+          <t>PERSON_LOST</t>
         </is>
       </c>
       <c r="C209" s="32" t="inlineStr">
         <is>
-          <t>명령 만료</t>
+          <t>추종 대상 놓침</t>
         </is>
       </c>
       <c r="D209" s="32" t="inlineStr">
         <is>
-          <t>실패·시간초과 결과</t>
+          <t>실패 FOLLOW_RESULT</t>
         </is>
       </c>
       <c r="E209" s="32" t="inlineStr">
         <is>
-          <t>expiresAt과 구분해 코드만 저장</t>
+          <t>고빈도 tracking 정보는 저장하지 않음</t>
         </is>
       </c>
     </row>
@@ -24534,22 +24554,22 @@
       </c>
       <c r="B210" s="32" t="inlineStr">
         <is>
-          <t>EXECUTION_TIMEOUT</t>
+          <t>COMMAND_EXPIRED</t>
         </is>
       </c>
       <c r="C210" s="32" t="inlineStr">
         <is>
-          <t>실행 시간초과</t>
+          <t>명령 만료</t>
         </is>
       </c>
       <c r="D210" s="32" t="inlineStr">
         <is>
-          <t>Robot 또는 Backend timeout</t>
+          <t>실패·시간초과 결과</t>
         </is>
       </c>
       <c r="E210" s="32" t="inlineStr">
         <is>
-          <t>늦은 STOPPED가 원인을 덮어쓰지 않음</t>
+          <t>expiresAt과 구분해 코드만 저장</t>
         </is>
       </c>
     </row>
@@ -24561,22 +24581,22 @@
       </c>
       <c r="B211" s="32" t="inlineStr">
         <is>
-          <t>SAFETY_STOP</t>
+          <t>EXECUTION_TIMEOUT</t>
         </is>
       </c>
       <c r="C211" s="32" t="inlineStr">
         <is>
-          <t>Robot 안전 정지</t>
+          <t>실행 시간초과</t>
         </is>
       </c>
       <c r="D211" s="32" t="inlineStr">
         <is>
-          <t>취소·실패 결과</t>
+          <t>Robot 또는 Backend timeout</t>
         </is>
       </c>
       <c r="E211" s="32" t="inlineStr">
         <is>
-          <t>terminal Robot mode는 SAFE_STOP</t>
+          <t>늦은 STOPPED가 원인을 덮어쓰지 않음</t>
         </is>
       </c>
     </row>
@@ -24588,49 +24608,49 @@
       </c>
       <c r="B212" s="32" t="inlineStr">
         <is>
-          <t>INTERNAL_ERROR</t>
+          <t>SAFETY_STOP</t>
         </is>
       </c>
       <c r="C212" s="32" t="inlineStr">
         <is>
-          <t>Robot 내부 오류</t>
+          <t>Robot 안전 정지</t>
         </is>
       </c>
       <c r="D212" s="32" t="inlineStr">
         <is>
-          <t>실패 FOLLOW_RESULT</t>
+          <t>취소·실패 결과</t>
         </is>
       </c>
       <c r="E212" s="32" t="inlineStr">
         <is>
-          <t>상세 예외 전문은 로그 경계에 둠</t>
+          <t>terminal Robot mode는 SAFE_STOP</t>
         </is>
       </c>
     </row>
     <row r="213" ht="26.39999961853027" customHeight="1">
       <c r="A213" s="32" t="inlineStr">
         <is>
-          <t>robot.occupancy_status / occupancy_event.resulting_occupancy</t>
+          <t>scenario.last_follow_reason_code</t>
         </is>
       </c>
       <c r="B213" s="32" t="inlineStr">
         <is>
-          <t>HOME</t>
+          <t>INTERNAL_ERROR</t>
         </is>
       </c>
       <c r="C213" s="32" t="inlineStr">
         <is>
-          <t>재실 확인</t>
+          <t>Robot 내부 오류</t>
         </is>
       </c>
       <c r="D213" s="32" t="inlineStr">
         <is>
-          <t>현관 IN 또는 발화 증거 적용 뒤 사용</t>
+          <t>실패 FOLLOW_RESULT</t>
         </is>
       </c>
       <c r="E213" s="32" t="inlineStr">
         <is>
-          <t>현재 스냅샷과 이벤트 결과를 같은 코드로 유지</t>
+          <t>상세 예외 전문은 로그 경계에 둠</t>
         </is>
       </c>
     </row>
@@ -24642,22 +24662,22 @@
       </c>
       <c r="B214" s="32" t="inlineStr">
         <is>
-          <t>AWAY</t>
+          <t>HOME</t>
         </is>
       </c>
       <c r="C214" s="32" t="inlineStr">
         <is>
-          <t>외출 확인</t>
+          <t>재실 확인</t>
         </is>
       </c>
       <c r="D214" s="32" t="inlineStr">
         <is>
-          <t>현관 OUT 증거 적용 뒤 사용</t>
+          <t>현관 IN 또는 발화 증거 적용 뒤 사용</t>
         </is>
       </c>
       <c r="E214" s="32" t="inlineStr">
         <is>
-          <t>침묵을 이상으로 오판하지 않게 함</t>
+          <t>현재 스냅샷과 이벤트 결과를 같은 코드로 유지</t>
         </is>
       </c>
     </row>
@@ -24669,49 +24689,49 @@
       </c>
       <c r="B215" s="32" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>AWAY</t>
         </is>
       </c>
       <c r="C215" s="32" t="inlineStr">
         <is>
-          <t>재실 불명</t>
+          <t>외출 확인</t>
         </is>
       </c>
       <c r="D215" s="32" t="inlineStr">
         <is>
-          <t>관측 전 또는 현관 하트비트 timeout 뒤 사용</t>
+          <t>현관 OUT 증거 적용 뒤 사용</t>
         </is>
       </c>
       <c r="E215" s="32" t="inlineStr">
         <is>
-          <t>HOME으로 낙관하지 않음</t>
+          <t>침묵을 이상으로 오판하지 않게 함</t>
         </is>
       </c>
     </row>
     <row r="216" ht="15" customHeight="1">
       <c r="A216" s="32" t="inlineStr">
         <is>
-          <t>occupancy_event.direction</t>
+          <t>robot.occupancy_status / occupancy_event.resulting_occupancy</t>
         </is>
       </c>
       <c r="B216" s="32" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="C216" s="32" t="inlineStr">
         <is>
-          <t>현관 안쪽 통과</t>
+          <t>재실 불명</t>
         </is>
       </c>
       <c r="D216" s="32" t="inlineStr">
         <is>
-          <t>귀가 이벤트에 사용</t>
+          <t>관측 전 또는 현관 하트비트 timeout 뒤 사용</t>
         </is>
       </c>
       <c r="E216" s="32" t="inlineStr">
         <is>
-          <t>방향 없는 재실 변화는 null</t>
+          <t>HOME으로 낙관하지 않음</t>
         </is>
       </c>
     </row>
@@ -24723,17 +24743,17 @@
       </c>
       <c r="B217" s="32" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C217" s="32" t="inlineStr">
         <is>
-          <t>현관 바깥쪽 통과</t>
+          <t>현관 안쪽 통과</t>
         </is>
       </c>
       <c r="D217" s="32" t="inlineStr">
         <is>
-          <t>외출 이벤트에 사용</t>
+          <t>귀가 이벤트에 사용</t>
         </is>
       </c>
       <c r="E217" s="32" t="inlineStr">
@@ -24745,27 +24765,27 @@
     <row r="218" ht="15" customHeight="1">
       <c r="A218" s="32" t="inlineStr">
         <is>
-          <t>occupancy_event.source</t>
+          <t>occupancy_event.direction</t>
         </is>
       </c>
       <c r="B218" s="32" t="inlineStr">
         <is>
-          <t>DOOR_SENSOR</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="C218" s="32" t="inlineStr">
         <is>
-          <t>현관 센서 확정</t>
+          <t>현관 바깥쪽 통과</t>
         </is>
       </c>
       <c r="D218" s="32" t="inlineStr">
         <is>
-          <t>문 통과 재실 변화에 사용</t>
+          <t>외출 이벤트에 사용</t>
         </is>
       </c>
       <c r="E218" s="32" t="inlineStr">
         <is>
-          <t>센서 reportedAt은 참고 시각</t>
+          <t>방향 없는 재실 변화는 null</t>
         </is>
       </c>
     </row>
@@ -24777,22 +24797,22 @@
       </c>
       <c r="B219" s="32" t="inlineStr">
         <is>
-          <t>SPEECH</t>
+          <t>DOOR_SENSOR</t>
         </is>
       </c>
       <c r="C219" s="32" t="inlineStr">
         <is>
-          <t>발화로 HOME 확정</t>
+          <t>현관 센서 확정</t>
         </is>
       </c>
       <c r="D219" s="32" t="inlineStr">
         <is>
-          <t>어르신 발화 감지 시 사용</t>
+          <t>문 통과 재실 변화에 사용</t>
         </is>
       </c>
       <c r="E219" s="32" t="inlineStr">
         <is>
-          <t>발화는 집 안 존재의 강한 증거</t>
+          <t>센서 reportedAt은 참고 시각</t>
         </is>
       </c>
     </row>
@@ -24804,49 +24824,49 @@
       </c>
       <c r="B220" s="32" t="inlineStr">
         <is>
-          <t>HEARTBEAT_TIMEOUT</t>
+          <t>SPEECH</t>
         </is>
       </c>
       <c r="C220" s="32" t="inlineStr">
         <is>
-          <t>현관 노드 통신 만료</t>
+          <t>발화로 HOME 확정</t>
         </is>
       </c>
       <c r="D220" s="32" t="inlineStr">
         <is>
-          <t>재실을 UNKNOWN으로 강등할 때 사용</t>
+          <t>어르신 발화 감지 시 사용</t>
         </is>
       </c>
       <c r="E220" s="32" t="inlineStr">
         <is>
-          <t>문 통과 사건이 아님</t>
+          <t>발화는 집 안 존재의 강한 증거</t>
         </is>
       </c>
     </row>
     <row r="221" ht="15" customHeight="1">
       <c r="A221" s="32" t="inlineStr">
         <is>
-          <t>care_record.notification_tier</t>
+          <t>occupancy_event.source</t>
         </is>
       </c>
       <c r="B221" s="32" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>HEARTBEAT_TIMEOUT</t>
         </is>
       </c>
       <c r="C221" s="32" t="inlineStr">
         <is>
-          <t>즉시 보호자 알림</t>
+          <t>현관 노드 통신 만료</t>
         </is>
       </c>
       <c r="D221" s="32" t="inlineStr">
         <is>
-          <t>응급·즉시 공유 사건</t>
+          <t>재실을 UNKNOWN으로 강등할 때 사용</t>
         </is>
       </c>
       <c r="E221" s="32" t="inlineStr">
         <is>
-          <t>T4는 이 컬럼에 저장하지 않음</t>
+          <t>문 통과 사건이 아님</t>
         </is>
       </c>
     </row>
@@ -24858,22 +24878,22 @@
       </c>
       <c r="B222" s="32" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="C222" s="32" t="inlineStr">
         <is>
-          <t>일간 요약</t>
+          <t>즉시 보호자 알림</t>
         </is>
       </c>
       <c r="D222" s="32" t="inlineStr">
         <is>
-          <t>추세·비응급 관찰 집계</t>
+          <t>응급·즉시 공유 사건</t>
         </is>
       </c>
       <c r="E222" s="32" t="inlineStr">
         <is>
-          <t>중복 발송은 summary_sent_at으로 방지</t>
+          <t>T4는 이 컬럼에 저장하지 않음</t>
         </is>
       </c>
     </row>
@@ -24885,20 +24905,47 @@
       </c>
       <c r="B223" s="32" t="inlineStr">
         <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C223" s="32" t="inlineStr">
+        <is>
+          <t>일간 요약</t>
+        </is>
+      </c>
+      <c r="D223" s="32" t="inlineStr">
+        <is>
+          <t>추세·비응급 관찰 집계</t>
+        </is>
+      </c>
+      <c r="E223" s="32" t="inlineStr">
+        <is>
+          <t>중복 발송은 summary_sent_at으로 방지</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="32" t="inlineStr">
+        <is>
+          <t>care_record.notification_tier</t>
+        </is>
+      </c>
+      <c r="B224" s="32" t="inlineStr">
+        <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="C223" s="32" t="inlineStr">
+      <c r="C224" s="32" t="inlineStr">
         <is>
           <t>시니어 동의 필요</t>
         </is>
       </c>
-      <c r="D223" s="32" t="inlineStr">
+      <c r="D224" s="32" t="inlineStr">
         <is>
           <t>민감 사실 공유 전 동의 흐름</t>
         </is>
       </c>
-      <c r="E223" s="32" t="inlineStr">
+      <c r="E224" s="32" t="inlineStr">
         <is>
           <t>권한·동의를 우회하지 않음</t>
         </is>

</xml_diff>